<commit_message>
Release SonarQube Profile Creator 1.2.0
</commit_message>
<xml_diff>
--- a/templates/sonarqube_rules_template.xlsx
+++ b/templates/sonarqube_rules_template.xlsx
@@ -413,148 +413,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>rule_key</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>target_profile</t>
+          <t>active</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>rule_key</t>
+          <t>severity</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>parent_profile</t>
+          <t>params</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>strategy</t>
+          <t>prioritizedRule</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>severity</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>params</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>prioritizedRule</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>project_key</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>set_default</t>
+          <t>note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>java</t>
+          <t>java:S1144</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PM Demo Java Profile</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>java:S1144</t>
+          <t>MAJOR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>extend_default</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>MAJOR</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
           <t>false</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>js</t>
+          <t>javascript:S1128</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PM Demo JS Profile</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>javascript:S1128</t>
-        </is>
-      </c>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>extend_default</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>